<commit_message>
added power sheet to schematic and started rough pcb placement
</commit_message>
<xml_diff>
--- a/Reference material/Data name conversion.xlsx
+++ b/Reference material/Data name conversion.xlsx
@@ -51,7 +51,7 @@
     <t>LV3</t>
   </si>
   <si>
-    <t>GND_DRAIN</t>
+    <t>DRAIN</t>
   </si>
   <si>
     <t>ATT2</t>
@@ -94,15 +94,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11.000000"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -117,87 +110,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="2">
     <border>
       <left style="none"/>
       <right style="none"/>
       <top style="none"/>
       <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="1"/>
-      </left>
-      <right style="medium">
-        <color theme="1"/>
-      </right>
-      <top style="medium">
-        <color theme="1"/>
-      </top>
-      <bottom style="medium">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="medium">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="medium">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="medium">
-        <color theme="1"/>
-      </right>
-      <top style="medium">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
       <diagonal style="none"/>
     </border>
     <border>
@@ -215,82 +133,13 @@
       </bottom>
       <diagonal style="none"/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="medium">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="medium">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="medium">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="medium">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="medium">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="2">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="8" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -818,85 +667,85 @@
       </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" ht="14.25">
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" ht="14.25">
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" ht="14.25">
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" ht="14.25">
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" ht="14.25">
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="1" t="s">
         <v>23</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="B3:D10" columnSort="0">
-    <sortCondition sortBy="value" descending="0" ref="C3:C10"/>
+  <sortState ref="B2:D9" columnSort="0">
+    <sortCondition sortBy="value" descending="0" ref="C2:C9"/>
   </sortState>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>